<commit_message>
Sjednica: true 45° orientation, 4 x 1x3 landscape stands, DC distribution
Plan north = true NE; wall names in true directions; S-01..S-03 with the rotated north arrow and 4 separate 1x3 landscape stands, 8 strip footings; M-01/E-01 with the -48 V DC distribution D1-D6; BOQ LOT 1/2 through fix_boq_sw_4x3l.py; 07-proracuni, 09 decision record and change log updated.
</commit_message>
<xml_diff>
--- a/bht-sjednica-final-review/TD-OUTPUT/3.1 PRILOG II TD - predmjer Sjednica Bileca.xlsx
+++ b/bht-sjednica-final-review/TD-OUTPUT/3.1 PRILOG II TD - predmjer Sjednica Bileca.xlsx
@@ -1374,14 +1374,14 @@
       <c r="B12" s="112" t="inlineStr">
         <is>
           <t>Isporuka i montaža nosive metalne konstrukcije (ground mount support) za prihvat fotonaponskih panela, karakteristika:
- - tip: CUSTOM IZRADA (izvan kataloga zbog opterećenja vjetrom, v. niže) — 3 nosača, svaki za 4 fotonaponska modula (2 reda × 2 kolone, portret); geometrija margina/prepusta preuzeta iz Huawei Standard A-Shaped Support 3.0 konvencije (PVM Tabela 4-20), ali poprečna greda izrađena po mjeri za 2 kolone modula, ne za kataloških 6
- - inklinacija: fiksno 45°, orijentacija JUG (azimut 180°). Nagib je zadržan zbog decembarskog prinosa — pri podnevnoj visini Sunca 23,6° na 42,94° N nagib 45° ostvaruje 93 % direktnog zračenja u odnosu na 85 % pri 35°, a decembar je mjerodavni mjesec za dimenzionisanje autonomnog sistema
- - gabariti PV polja po nosaču (2 reda × 2 modula, portret): širina polja 2305 mm (poprečna greda 2918 mm, bočni prepust 306,5 mm), dužina polja po nagibu 4576 mm (2 × 2278 mm, nepromijenjeno), horizontalna projekcija 3236 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +3,74 m od nivoa terena
- - smještaj: nosači se temelje IZVAN ograđenog platoa, južno od ograde, u pojasu širine cca 1950 mm; odmak od ograde ponuđač utvrđuje pri poziciranju nosača tako da ravan panela nigdje ne dodiruje ogradu; gornja (sjeverna) ivica panela je 1,64 m iznad kote ograde h=2,10 m. Ponuđač provjerava da konstrukcija u cijelosti ostaje unutar zakupljene parcele 16,00 × 9,40 m
- - MJERODAVNO OPTEREĆENJE VJETROM: qp ≥ 1,20 kN/m² (udar 3 s ≈ 45 m/s) prema ovjerenoj projektnoj dokumentaciji lokacije i BAS EN 1991-1-4 sa BiH nacionalnim aneksom, uz primjenu faktora orografije za izloženi planinski vrh na 1076 m n.v. Koeficijent sile cf ≥ 1,5 pri 45° prema EN 1991-1-4 §7.3, osim ako se proračunom dokaže drugačije. Površina izloženosti vjetru 10,55 m² po nosaču (2305 × 4576 mm). Projektne sile po nosaču (GSN, γQ=1,5 / γG,fav=0,9): podizanje ≥18,1 kN, horizontalna sila ≥13,4 kN, moment prevrtanja ≥42,6 kNm. Mjerodavni su podizanje (uplift) i prevrtanje, a ne nosivost tla. NAPOMENA: kataloški nosač tipa A ima deklarisanu otpornost 31 m/s (0,52 kN/m²) pri 45° i 40 m/s (0,87 kN/m²) pri 15°/25°, što je ISPOD opterećenja ovog lokaliteta čak i za manje polje; Ponuđač je stoga dužan ponuditi konstrukciju dimenzionisanu i dokazanu za stvarno opterećenje lokaliteta, uz pisanu potvrdu proizvođača za konkretnu lokaciju (planinski vrh) ako se ipak nudi kataloški proizvod
+ - tip: CUSTOM IZRADA (izvan kataloga zbog opterećenja vjetrom, v. niže) — 4 odvojena nosača u jednom nizu, svaki za 3 fotonaponska modula (3 reda × 1 kolona, položeno); odvojeni nosači umjesto jednog velikog polja smanjuju silu vjetra po konstrukciji (zahtjev Naručioca); geometrija margina/prepusta preuzeta iz Huawei Standard A-Shaped Support 3.0 konvencije (PVM Tabela 4-20), ali poprečna greda izrađena po mjeri za 1 kolonu položenih modula, ne za kataloških 6
+ - inklinacija: fiksno 45°, orijentacija JUGOZAPAD (azimut 225°), niz paralelan sa jugozapadnom ogradom (Naručilac 11.09.2026). Nagib je zadržan zbog decembarskog prinosa — pri podnevnoj visini Sunca 23,6° na 42,94° N nagib 45° ostvaruje 93 % direktnog zračenja u odnosu na 85 % pri 35°, a decembar je mjerodavni mjesec za dimenzionisanje autonomnog sistema
+ - gabariti PV polja po nosaču (3 reda × 1 modul, položeno): širina polja 2278 mm (poprečna greda 2891 mm, bočni prepust 306,5 mm), dužina polja po nagibu 3442 mm (3 × 1134 mm + 2 × 20 mm), horizontalna projekcija 2434 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +2,93 m od nivoa terena; razmak između nosača 400 mm, dužina niza 10 312 mm
+ - smještaj: nosači se temelje IZVAN ograđenog platoa, jugozapadno od ograde (JZ strana), cca 0,40 m od ograde; odmak od ograde ponuđač utvrđuje pri poziciranju nosača tako da ravan panela nigdje ne dodiruje ogradu; gornja (sjeveroistočna) ivica panela je 0,83 m iznad kote ograde h=2,10 m. Ponuđač provjerava da konstrukcija u cijelosti ostaje unutar zakupljene parcele 16,00 × 9,40 m
+ - MJERODAVNO OPTEREĆENJE VJETROM: qp ≥ 1,20 kN/m² (udar 3 s ≈ 45 m/s) prema ovjerenoj projektnoj dokumentaciji lokacije i BAS EN 1991-1-4 sa BiH nacionalnim aneksom, uz primjenu faktora orografije za izloženi planinski vrh na 1076 m n.v. Koeficijent sile cf ≥ 1,5 pri 45° prema EN 1991-1-4 §7.3, osim ako se proračunom dokaže drugačije. Površina izloženosti vjetru 7,84 m² po nosaču (2278 × 3442 mm). Projektne sile po nosaču (GSN, γQ=1,5 / γG,fav=0,9): podizanje ≥13,3 kN, horizontalna sila ≥10,0 kN, moment prevrtanja ≥25,7 kNm. Mjerodavni su podizanje (uplift) i prevrtanje, a ne nosivost tla. NAPOMENA: kataloški nosač tipa A ima deklarisanu otpornost 31 m/s (0,52 kN/m²) pri 45° i 40 m/s (0,87 kN/m²) pri 15°/25°, što je ISPOD opterećenja ovog lokaliteta čak i za manje polje; Ponuđač je stoga dužan ponuditi konstrukciju dimenzionisanu i dokazanu za stvarno opterećenje lokaliteta, uz pisanu potvrdu proizvođača za konkretnu lokaciju (planinski vrh) ako se ipak nudi kataloški proizvod
  - materijal i izrada: konstrukcijski čelik S275JR (S355JR za stubove) prema EN 10025-2, šuplji profili prema EN 10219 — stubovi min. RHS 80×80×4, rigle min. RHS 60×40×3, ili bilo koji presjek za koji se proračunom dokaže najmanje jednak otporni moment; antikorozivna zaštita vrućim cinčanjem prema EN ISO 1461 min. 70 µm lokalno / 85 µm srednje (klasa korozivnosti C4); zavarivanje prema EN 1090-2 klasa izvedbe EXC2; CE označavanje i izjava o svojstvima prema EN 1090-1; konstrukcijski vijci M16 klase 8.8 prema EN 15048, pričvrsni pribor modula A2/A4 nehrđajući
  - spojni pribor: nehrđajući čelik A2/A4
- - uključeno ožičenje i povezivanje panela do PVDB distribucije preko po-string DC odvodnika prenapona (v. crtež E-01): 12 modula se povezuje u DVA STRINGA po 6 modula (string 1 — nosači PV-1 i PV-2; string 2 — nosači PV-2 i PV-3), po jedan string na svaku od dvije rute PVDB ormara</t>
+ - uključeno ožičenje i povezivanje panela do PVDB distribucije preko po-string DC odvodnika prenapona (v. crtež E-01): 12 modula se povezuje u DVA STRINGA po 6 modula (string 1 — nosači PV-1 i PV-2; string 2 — nosači PV-3 i PV-4), po jedan string na svaku od dvije rute PVDB ormara</t>
         </is>
       </c>
       <c r="C12" s="113" t="inlineStr">
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="D12" s="113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" s="114" t="n"/>
       <c r="F12" s="114">
@@ -1409,9 +1409,9 @@
           <t>Isporuka i ugradnja sistema sidrenja nosive konstrukcije iz Tačke 1.1 u stijenu/beton, hemijskim (epoksidnim) ankerima.
  - tip: hemijski (epoksidni/vinilesterski) anker M16 ili M20 sa ETA odobrenjem za ugradnju u beton i/ili stijenu, vruće cinčan ili nehrđajući A4
  - broj: najmanje 2 ankera po temeljnoj traci, odnosno 4 ankera po nosaču (minimum 2 po traci zbog redundanse)
- - nosivost: karakteristična sila čupanja ≥30 kN po ankeru; dubina ugradnje prema ETA za konkretnu podlogu. Ukupna projektna sila podizanja po nosaču ≥18,1 kN (GSN); sila po traci od momenta prevrtanja ≥26,6 kN pri razmaku traka 1600 mm
+ - nosivost: karakteristična sila čupanja ≥30 kN po ankeru; dubina ugradnje prema ETA za konkretnu podlogu. Ukupna projektna sila podizanja po nosaču ≥13,3 kN (GSN); sila po traci od momenta prevrtanja ≥16,1 kN pri razmaku traka 1600 mm
  - dokazivanje: ispitivanje čupanjem (pull-out test) na najmanje 10 % ugrađenih ankera, minimalno 2 po nosaču, do 1,5 × projektne sile, uz zapisnik ovjeren od nadzornog organa
- - alternativa: livena U-anker sidra M16, dužine 320 mm, razmaka krakova 180 mm, sa pločama 50×50 mm i dvostrukim maticama, dozvoljena su SAMO uz gravitacioni temelj zapremine ≥0,75 m³ po nosaču (tendovano 0,81 m³ po nosaču, v. Tačku 2.3) — momenat prevrtanja i dalje zahtijeva provjeru lokalnog istezanja trake, ne samo ukupne mase</t>
+ - alternativa: livena U-anker sidra M16, dužine 320 mm, razmaka krakova 180 mm, sa pločama 50×50 mm i dvostrukim maticama, dozvoljena su SAMO uz gravitacioni temelj iz Tačke 2.3 (dvije trake po nosaču, najmanje 0,74 m³ po traci; tendovano 1,053 m³ po traci) — momenat prevrtanja i dalje zahtijeva provjeru lokalnog istezanja trake, ne samo ukupne mase</t>
         </is>
       </c>
       <c r="C13" s="113" t="inlineStr">
@@ -1420,7 +1420,7 @@
         </is>
       </c>
       <c r="D13" s="113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" s="114" t="n"/>
       <c r="F13" s="114">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B15" s="116" t="inlineStr">
         <is>
-          <t>Uzemljenje nosivih konstrukcija: povezivanje sva tri nosača na postojeći prstenasti uzemljivač lokacije bakarnim užetom presjeka 50 mm² sa izolacijom otpornom na UV zračenje i ukopavanje, preko priključnih stezaljki na konstrukciji i bimetalnih (Cu/Fe-Zn) ukrsnih komada radi sprječavanja galvanske korozije. Presjek prema EN 62305-3, Tabela 7, za odvođenje atmosferskog pražnjenja. Kontinuitet svih spojeva ≤0,1 Ω, ukupni otpor uzemljenja ≤10 Ω. DC kablovi se polažu na razmaku ≥0,5 m od odvoda gromobranske instalacije (Huawei §4.1.3).</t>
+          <t>Uzemljenje nosivih konstrukcija: povezivanje sva četiri nosača na postojeći prstenasti uzemljivač lokacije bakarnim užetom presjeka 50 mm² sa izolacijom otpornom na UV zračenje i ukopavanje, preko priključnih stezaljki na konstrukciji i bimetalnih (Cu/Fe-Zn) ukrsnih komada radi sprječavanja galvanske korozije. Presjek prema EN 62305-3, Tabela 7, za odvođenje atmosferskog pražnjenja. Kontinuitet svih spojeva ≤0,1 Ω, ukupni otpor uzemljenja ≤10 Ω. DC kablovi se polažu na razmaku ≥0,5 m od odvoda gromobranske instalacije (Huawei §4.1.3).</t>
         </is>
       </c>
       <c r="C15" s="117" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="D15" s="117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="118" t="n"/>
       <c r="F15" s="118">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B20" s="129" t="inlineStr">
         <is>
-          <t>Iskop zemlje/stijene IV-V kategorije za temeljne trake nosača, do donje ivice podložnog betona. Rov širine 550 mm, dubine 950 mm, dužine 3300 mm. 3 nosača × 2 trake × 1,725 m3</t>
+          <t>Iskop zemlje/stijene IV-V kategorije za temeljne trake nosača, do donje ivice podložnog betona. Rov širine 500 mm, dubine 950 mm, dužine 2600 mm. 4 nosača × 2 trake × 1,235 m3</t>
         </is>
       </c>
       <c r="C20" s="130" t="inlineStr">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="D20" s="130" t="n">
-        <v>10.35</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E20" s="131" t="n"/>
       <c r="F20" s="131">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="B21" s="132" t="inlineStr">
         <is>
-          <t>Zatrpavanje preostalog dijela rova zemljom od iskopa uz nabijanje u slojevima. Traka je pune dubine, pa se zatrpava samo klin uz kosinu rova. 3 nosača × 2 trake × 0,149 m3</t>
+          <t>Zatrpavanje preostalog dijela rova zemljom od iskopa uz nabijanje u slojevima. Traka je pune dubine, pa se zatrpava samo klin uz kosinu rova. 4 nosača × 2 trake × 0,117 m3</t>
         </is>
       </c>
       <c r="C21" s="130" t="inlineStr">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="D21" s="130" t="n">
-        <v>0.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E21" s="131" t="n"/>
       <c r="F21" s="131">
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D22" s="130" t="n">
-        <v>9.449999999999999</v>
+        <v>8.94</v>
       </c>
       <c r="E22" s="131" t="n"/>
       <c r="F22" s="131">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="B23" s="129" t="inlineStr">
         <is>
-          <t>Nabavka materijala, transport i ugradnja podložnog betona C12/15 ispod temeljnih traka, prema zahtjevima proizvođača. 3 nosača × 2 trake × 0,091 m3</t>
+          <t>Nabavka materijala, transport i ugradnja podložnog betona C12/15 ispod temeljnih traka, prema zahtjevima proizvođača. 4 nosača × 2 trake × 0,065 m3</t>
         </is>
       </c>
       <c r="C23" s="130" t="inlineStr">
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="D23" s="130" t="n">
-        <v>0.54</v>
+        <v>0.52</v>
       </c>
       <c r="E23" s="131" t="n"/>
       <c r="F23" s="131">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B24" s="129" t="inlineStr">
         <is>
-          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C30/37 klase izloženosti XC4 + XF3 prema BAS EN 206 (aerant 4–6 %, Dmax 16, konzistencija S3), uz upotrebu oplate i njegovanje betona. Armatura B500B, zaštitni sloj ≥50 mm, prema ovjerenom statičkom proračunu iz Tačke 1.3. Obračun po m³ ugrađenog betona. Traka 450 mm (gore) / 550 mm (dolje) × 3300 mm, PUNE dubine 900 mm = 1,485 m³ po traci. 3 nosača × 2 trake × 1,485 m³
+          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C30/37 klase izloženosti XC4 + XF3 prema BAS EN 206 (aerant 4–6 %, Dmax 16, konzistencija S3), uz upotrebu oplate i njegovanje betona. Armatura B500B, zaštitni sloj ≥50 mm, prema ovjerenom statičkom proračunu iz Tačke 1.3. Obračun po m³ ugrađenog betona. Traka 400 mm (gore) / 500 mm (dolje) × 2600 mm, PUNE dubine 900 mm = 1,053 m³ po traci. 4 nosača × 2 trake × 1,053 m³
 BETON I ARMATURA: beton klase C30/37, klase izloženosti XC4 + XF3 prema BAS EN 206, sa aerantom 4–6 %, Dmax 16, konzistencija S3; podložni beton C12/15 d=50 mm; armatura B500B, zaštitni sloj ≥50 mm. Klasa XF3 je mjerodavna zbog cikličnog smrzavanja i odmrzavanja u vlažnom stanju na 1076 m n.v. Temeljna spojnica mora biti ispod dubine smrzavanja za lokalitet, koju Ponuđač navodi u ponudi. Dubina 900 mm je tenderska osnova i mjerodavna je za ponudu; konačnu dubinu i armaturu potvrđuje ovjereni statički proračun iz Tačke 1.3. Traka se betonira punom dubinom rova — vlastita težina trake je dio dokaza sigurnosti na podizanje i prevrtanje.</t>
         </is>
       </c>
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D24" s="130" t="n">
-        <v>8.91</v>
+        <v>8.42</v>
       </c>
       <c r="E24" s="131" t="n"/>
       <c r="F24" s="131">
@@ -2150,8 +2150,8 @@
       <c r="B16" s="161" t="inlineStr">
         <is>
           <t>Isporuka i montaža automatskog DEA opisanog pod Tačkom 3.1 u postojeći kontejner, u skid izvedbi, na antivibracionim gumeno-metalnim osloncima (min. 4 kom, vlastita frekvencija ≤8 Hz, statički progib ≥5 mm), postavljenim između skida i roštilja iz Tačke 4.3, sa pripremom za pričvršćenje za podlogu. Stavka obuhvata i nabavnu vrijednost agregata iz Tačke 3.1.
- - PRISTUP: unos kroz kapiju na sredini istočne strane ograde (svijetla širina cca 1,00 m) i ulazna vrata kontejnera 900 × 2000 mm; ponuđač bira način unosa i dužan je u ponudi potvrditi izvodljivost
- - SERVISNI PROSTOR ( prema crtežu M-01): agregat se postavlja CENTRIRANO u slobodnom prostoru kontejnera, sa najmanje 720 mm sa JUŽNE i 720 mm sa SJEVERNE strane (520 mm na dijelu gdje je GRO) te 1155 mm sa ISTOČNE strane. Sa ZAPADNE strane je hladnjak, koji izduvava u kanal kroz zid i ne servisira se s te strane
+ - PRISTUP: unos kroz kapiju na sredini jugoistočne strane ograde (svijetla širina cca 1,00 m) i ulazna vrata kontejnera 900 × 2000 mm; ponuđač bira način unosa i dužan je u ponudi potvrditi izvodljivost
+ - SERVISNI PROSTOR ( prema crtežu M-01): agregat se postavlja CENTRIRANO u slobodnom prostoru kontejnera, sa najmanje 720 mm sa JUGOZAPADNE i 720 mm sa SJEVEROISTOČNE strane (520 mm na dijelu gdje je GRO) te 1155 mm sa JUGOISTOČNE strane. Sa SJEVEROZAPADNE strane je hladnjak, koji izduvava u kanal kroz zid i ne servisira se s te strane
  - dimenzije skida prilagoditi raspoloživom prostoru
  - dozvoljeni nivo buke izvan kontejnera &lt;68 dBA pri opterećenju 75 % na 7 m, režim Standby
  - taster EMERGENCY STOP uz ulazna vrata kontejnera</t>
@@ -2180,7 +2180,7 @@
       <c r="B17" s="161" t="inlineStr">
         <is>
           <t>Isporuka, montaža i povezivanje dvoplašnog spremnika dizel goriva zapremine 500 l (0,5 m³), od čeličnog lima, sa svim spojnim priborom, cjevovodima i armaturama. Zapremina spremnika nije predmet varijantnih rješenja i ne umanjuje se ni u slučaju ojačanja poda iz Tačke 4.3.
- - referentne dimenzije 1050 × 600 × 1310 mm, masa prazan 170 kg (pun ≈590 kg); smještaj u JUGOISTOČNI ugao kontejnera, prema crtežu M-01
+ - referentne dimenzije 1050 × 600 × 1310 mm, masa prazan 170 kg (pun ≈590 kg); smještaj u JUŽNI ugao kontejnera (uz JZ i JI zid), prema crtežu M-01
  - odušna cijev izvedena IZVAN kontejnera, otvor zaštićen metalnom mrežicom; odzračni cjevovod od čeličnih bešavnih cijevi prema DIN 2448 sa odzračnim ventilom tip AT
  - priključak za punjenje sa zatvaračem, izveden na vanjskoj strani kontejnera; obezbijediti prilaz autocisterne, a na pretakalištu ugraditi uređaj za odvođenje statičkog elektriciteta
  - priključak za pražnjenje sa zatvaračem i priključkom za crijevo
@@ -2264,8 +2264,8 @@
       </c>
       <c r="B20" s="161" t="inlineStr">
         <is>
-          <t>Izrada i montaža limenog kanala za odvod toplog zraka sa agregata, od pocinčanog lima d=1 mm, sa prirubnicama 30 × 1,5 mm, komplet sa fazonskim komadima i ovjesnim priborom. Kanal je PRELAZNI KOMAD od prirubnice hladnjaka do žaluzine 600 × 600 mm kroz ZAPADNI zid; hladnjak je 60 mm od zida, pa je razvijena površina ≈1,0 m². Stvarnu mjeru uzeti na licu mjesta prema ponuđenom agregatu.
-RASPORED (OBAVEZNO, prema crtežu M-01): kanal se vodi najkraćim putem od radijatora kroz ZAPADNI zid kontejnera do izlazne žaluzine iz Tačke 4.6.</t>
+          <t>Izrada i montaža limenog kanala za odvod toplog zraka sa agregata, od pocinčanog lima d=1 mm, sa prirubnicama 30 × 1,5 mm, komplet sa fazonskim komadima i ovjesnim priborom. Kanal je PRELAZNI KOMAD od prirubnice hladnjaka do žaluzine 600 × 600 mm kroz SJEVEROZAPADNI (SZ) zid; hladnjak je 60 mm od zida, pa je razvijena površina ≈1,0 m². Stvarnu mjeru uzeti na licu mjesta prema ponuđenom agregatu.
+RASPORED (OBAVEZNO, prema crtežu M-01): kanal se vodi najkraćim putem od radijatora kroz SJEVEROZAPADNI (SZ) zid kontejnera do izlazne žaluzine iz Tačke 4.6.</t>
         </is>
       </c>
       <c r="C20" s="128" t="inlineStr">
@@ -2291,7 +2291,7 @@
       <c r="B21" s="161" t="inlineStr">
         <is>
           <t>Isporuka i montaža fiksne žaluzine na kraju kanala za odvod toplog zraka, dimenzija 600 × 600 mm, sa zaštitnom mrežicom, komplet sa montažnim materijalom.
-RASPORED (OBAVEZNO, prema crtežu M-01): žaluzina se ugrađuje u ZAPADNI zid kontejnera, na osi radijatora agregata. Topli zrak i izduv se NE smiju izbacivati prema SJEVERNOJ strani, gdje se nalaze postojeći vanjski ormari ICC360-HA1-C1 i MTS9302A i gdje se nalazi usis svježeg zraka.</t>
+RASPORED (OBAVEZNO, prema crtežu M-01): žaluzina se ugrađuje u SJEVEROZAPADNI (SZ) zid kontejnera, na osi radijatora agregata. Topli zrak i izduv se NE smiju izbacivati prema SJEVEROISTOČNOJ (SI) strani, gdje se nalaze postojeći vanjski ormari ICC360-HA1-C1 i MTS9302A i gdje se nalazi usis svježeg zraka.</t>
         </is>
       </c>
       <c r="C21" s="128" t="inlineStr">
@@ -2317,7 +2317,7 @@
       <c r="B22" s="161" t="inlineStr">
         <is>
           <t>Isporuka i montaža vanjske fiksne žaluzine za dovod svježeg zraka, dimenzija 500 × 700 mm, sa zaštitnom mrežicom. Žaluzine postaviti tako da se spriječi ulaz vode u kontejner prilikom padavina.
-RASPORED (OBAVEZNO, prema crtežu M-01): žaluzina se ugrađuje u SJEVERNI zid kontejnera, na istočnom kraju, sa donjom ivicom na cca 0,30 m od poda. Sjeverna strana je zasjenjena i daje najhladniji usisni zrak, čime se poboljšava hlađenje agregata. Žaluzina se postavlja istočno od vanjskih ormara ICC360-HA1-C1/MTS9302A kako se ne bi usisavao topli zrak sa njih. Prostorna udaljenost od izduva i od odušne cijevi spremnika ≥3 m. Nije dozvoljeno izvesti dovod zraka kroz ulazna vrata.</t>
+RASPORED (OBAVEZNO, prema crtežu M-01): žaluzina se ugrađuje u SJEVEROISTOČNI (SI) zid kontejnera, na jugoistočnom kraju, sa donjom ivicom na cca 0,30 m od poda. Sjeveroistočna strana je zasjenjena veći dio dana i daje najhladniji usisni zrak, čime se poboljšava hlađenje agregata. Žaluzina se postavlja jugoistočno od vanjskih ormara ICC360-HA1-C1/MTS9302A kako se ne bi usisavao topli zrak sa njih. Prostorna udaljenost od izduva i od odušne cijevi spremnika ≥3 m. Nije dozvoljeno izvesti dovod zraka kroz ulazna vrata.</t>
         </is>
       </c>
       <c r="C22" s="128" t="inlineStr">
@@ -2343,7 +2343,7 @@
       <c r="B23" s="161" t="inlineStr">
         <is>
           <t>Isporuka i montaža aksijalnog EC ventilatora 48 V DC za prinudnu ventilaciju prostora agregata, kapaciteta 1200 m³/h, Ø315 mm, napajanog iz DC razvoda −48 V (Tačka 5.16), sa termostatskim upravljanjem. Ventilator radi prema termostatu dok agregat miruje; za vrijeme rada agregata kontroler agregata ga isključuje. Minimalna potrebna ventilacija prostora iznosi 120 m³/h (6 izmjena zraka na sat).
-RASPORED (prema crtežu M-01): ventilator se ugrađuje u ISTOČNI zid kontejnera, u gornjoj zoni (donja ivica cca 1,75 m), sjeverno od ulaznih vrata.</t>
+RASPORED (prema crtežu M-01): ventilator se ugrađuje u JUGOISTOČNI (JI) zid kontejnera, u gornjoj zoni (donja ivica cca 1,75 m), sjeveroistočno od ulaznih vrata.</t>
         </is>
       </c>
       <c r="C23" s="128" t="inlineStr">
@@ -2394,7 +2394,7 @@
       <c r="B25" s="161" t="inlineStr">
         <is>
           <t>Isporuka i montaža sistema za odvod izduvnih gasova: čelična cijev NO 50 mm sa ispušnim loncem (prigušivačem), izvedena izvan kontejnera i završena IZNAD KROVA, usmjereno naviše, sa kapom protiv upada padavina. Na kraju izduvne cijevi postaviti HVATAČ ISKRI. Dužine: od elastičnog umetka do prigušivača, sa jednim lukom 90°, 1 m; od prigušivača do izlaza iznad krova, do 4 m. Komplet sa elastičnim umetkom, lukovima i montažnim materijalom.
-TRASA: fleksibilni spoj i prigušivač neposredno iza motora, uspon uz ZAPADNI zid kontejnera, završetak IZNAD KROVA usmjeren naviše, sa hvatačem iskri.
+TRASA: fleksibilni spoj i prigušivač neposredno iza motora, uspon uz SJEVEROZAPADNI (SZ) zid kontejnera, završetak IZNAD KROVA usmjeren naviše, sa hvatačem iskri.
 NO 50: sa agregatom 18 kVA protok izduvnih gasova je 192 m³/h pri 413 °C, brzina 27,2 m/s (ispod uobičajenih 30 m/s), protutlak ≈1,9 kPa uz dozvoljenih 10,2 kPa.</t>
         </is>
       </c>

</xml_diff>